<commit_message>
DTR FEB16-28 and JAN16-31 correction
</commit_message>
<xml_diff>
--- a/DTR/2026/JAN16-31/AscendionNew_35311_John_01-16-2026.xlsx
+++ b/DTR/2026/JAN16-31/AscendionNew_35311_John_01-16-2026.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="121">
   <si>
     <t xml:space="preserve">Client Name</t>
   </si>
@@ -736,24 +736,24 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="116">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -761,31 +761,31 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -793,39 +793,39 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
@@ -837,7 +837,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -845,7 +845,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -853,35 +853,35 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="true">
+    <xf numFmtId="171" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -889,19 +889,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="174" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="175" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -909,103 +909,103 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1013,19 +1013,19 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1033,19 +1033,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1057,7 +1057,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="10" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="10" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1069,7 +1069,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1093,19 +1093,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="177" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="177" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="178" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="178" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="179" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="179" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1117,6 +1117,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
@@ -1129,19 +1133,19 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1161,27 +1165,27 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1189,11 +1193,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1211,54 +1215,7 @@
     <cellStyle name="Normal 2 2" xfId="23"/>
     <cellStyle name="Normal 3" xfId="24"/>
   </cellStyles>
-  <dxfs count="8">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9C0006"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB3A2C7"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC3D69B"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2461,7 +2418,9 @@
       <c r="K14" s="79"/>
       <c r="L14" s="84"/>
       <c r="M14" s="79"/>
-      <c r="N14" s="79"/>
+      <c r="N14" s="79" t="s">
+        <v>2</v>
+      </c>
       <c r="O14" s="85"/>
       <c r="P14" s="85"/>
       <c r="Q14" s="86"/>
@@ -4281,7 +4240,9 @@
       <c r="K18" s="94"/>
       <c r="L18" s="82"/>
       <c r="M18" s="94"/>
-      <c r="N18" s="79"/>
+      <c r="N18" s="79" t="s">
+        <v>2</v>
+      </c>
       <c r="O18" s="85"/>
       <c r="P18" s="94"/>
       <c r="Q18" s="86"/>
@@ -4743,7 +4704,9 @@
       <c r="K19" s="79"/>
       <c r="L19" s="84"/>
       <c r="M19" s="79"/>
-      <c r="N19" s="79"/>
+      <c r="N19" s="79" t="s">
+        <v>2</v>
+      </c>
       <c r="O19" s="85"/>
       <c r="P19" s="79"/>
       <c r="Q19" s="86"/>
@@ -5205,7 +5168,9 @@
       <c r="K20" s="79"/>
       <c r="L20" s="84"/>
       <c r="M20" s="79"/>
-      <c r="N20" s="79"/>
+      <c r="N20" s="79" t="s">
+        <v>2</v>
+      </c>
       <c r="O20" s="85"/>
       <c r="P20" s="79"/>
       <c r="Q20" s="86"/>
@@ -5667,7 +5632,9 @@
       <c r="K21" s="79"/>
       <c r="L21" s="84"/>
       <c r="M21" s="79"/>
-      <c r="N21" s="79"/>
+      <c r="N21" s="79" t="s">
+        <v>2</v>
+      </c>
       <c r="O21" s="85"/>
       <c r="P21" s="79"/>
       <c r="Q21" s="86"/>
@@ -6122,9 +6089,7 @@
       <c r="N22" s="79"/>
       <c r="O22" s="85"/>
       <c r="P22" s="79"/>
-      <c r="Q22" s="86" t="s">
-        <v>111</v>
-      </c>
+      <c r="Q22" s="95"/>
       <c r="R22" s="87" t="n">
         <f aca="false">IF(AND(C22="Normal",I22&gt;0),(8-S22),0)-IF(AND(C22="Normal",OR(C23="Special Holiday",C23="Working - Legal Holiday on RD",C23="Working - Special Holiday on RD",C23="Legal Holiday",C23="Legal Holiday on RD",C23="Special Holiday on RD")),BN22,0)+IF(AND(OR(C22="Normal",C22="Leave",C22="Rest Day"),OR(C21="Special Holiday",C21="Working - Legal Holiday on RD",C21="Working - Special Holiday on RD",C21="Legal Holiday")),BN21,0)</f>
         <v>0</v>
@@ -7028,7 +6993,9 @@
       <c r="N24" s="79"/>
       <c r="O24" s="85"/>
       <c r="P24" s="79"/>
-      <c r="Q24" s="86"/>
+      <c r="Q24" s="86" t="s">
+        <v>111</v>
+      </c>
       <c r="R24" s="87" t="n">
         <f aca="false">IF(AND(C24="Normal",I24&gt;0),(8-S24),0)-IF(AND(C24="Normal",OR(C25="Special Holiday",C25="Working - Legal Holiday on RD",C25="Working - Special Holiday on RD",C25="Legal Holiday",C25="Legal Holiday on RD",C25="Special Holiday on RD")),BN24,0)+IF(AND(OR(C24="Normal",C24="Leave",C24="Rest Day"),OR(C23="Special Holiday",C23="Working - Legal Holiday on RD",C23="Working - Special Holiday on RD",C23="Legal Holiday")),BN23,0)</f>
         <v>0</v>
@@ -7483,11 +7450,13 @@
         <f aca="false">IFERROR(IF(N25="Strict",IF(C25="Normal",IFERROR(IF((HOUR(IF(AQ25&lt;=AR25,BB25-AR25,BB25-AQ25))+MINUTE(IF(AQ25&lt;=AR25,BB25-AR25,BB25-AQ25))/60)&gt;=6,HOUR(IF(AQ25&lt;=AR25,BB25-AR25,BB25-AQ25))+MINUTE(IF(AQ25&lt;=AR25,BB25-AR25,BB25-AQ25))/60-1,HOUR(IF(AQ25&lt;=AR25,BB25-AR25,BB25-AQ25))+MINUTE(IF(AQ25&lt;=AR25,BB25-AR25,BB25-AQ25))/60),0),0),IF(N25="Flexi",IF(C25="Normal",IF((HOUR(BB25-AR25)+MINUTE(BB25-AR25)/60)&gt;=6,(HOUR(BB25-AR25)+MINUTE(BB25-AR25)/60)-1,(HOUR(BB25-AR25)+MINUTE(BB25-AR25)/60)),0),0)),0)</f>
         <v>0</v>
       </c>
-      <c r="J25" s="95"/>
+      <c r="J25" s="96"/>
       <c r="K25" s="79"/>
       <c r="L25" s="82"/>
       <c r="M25" s="79"/>
-      <c r="N25" s="79"/>
+      <c r="N25" s="79" t="s">
+        <v>2</v>
+      </c>
       <c r="O25" s="85"/>
       <c r="P25" s="79"/>
       <c r="Q25" s="86"/>
@@ -7945,11 +7914,13 @@
         <f aca="false">IFERROR(IF(N26="Strict",IF(C26="Normal",IFERROR(IF((HOUR(IF(AQ26&lt;=AR26,BB26-AR26,BB26-AQ26))+MINUTE(IF(AQ26&lt;=AR26,BB26-AR26,BB26-AQ26))/60)&gt;=6,HOUR(IF(AQ26&lt;=AR26,BB26-AR26,BB26-AQ26))+MINUTE(IF(AQ26&lt;=AR26,BB26-AR26,BB26-AQ26))/60-1,HOUR(IF(AQ26&lt;=AR26,BB26-AR26,BB26-AQ26))+MINUTE(IF(AQ26&lt;=AR26,BB26-AR26,BB26-AQ26))/60),0),0),IF(N26="Flexi",IF(C26="Normal",IF((HOUR(BB26-AR26)+MINUTE(BB26-AR26)/60)&gt;=6,(HOUR(BB26-AR26)+MINUTE(BB26-AR26)/60)-1,(HOUR(BB26-AR26)+MINUTE(BB26-AR26)/60)),0),0)),0)</f>
         <v>0</v>
       </c>
-      <c r="J26" s="95"/>
+      <c r="J26" s="96"/>
       <c r="K26" s="79"/>
       <c r="L26" s="82"/>
       <c r="M26" s="79"/>
-      <c r="N26" s="79"/>
+      <c r="N26" s="79" t="s">
+        <v>2</v>
+      </c>
       <c r="O26" s="85"/>
       <c r="P26" s="79"/>
       <c r="Q26" s="86"/>
@@ -8411,7 +8382,9 @@
       <c r="K27" s="79"/>
       <c r="L27" s="84"/>
       <c r="M27" s="79"/>
-      <c r="N27" s="79"/>
+      <c r="N27" s="79" t="s">
+        <v>2</v>
+      </c>
       <c r="O27" s="85"/>
       <c r="P27" s="79"/>
       <c r="Q27" s="86"/>
@@ -8873,7 +8846,9 @@
       <c r="K28" s="79"/>
       <c r="L28" s="84"/>
       <c r="M28" s="79"/>
-      <c r="N28" s="79"/>
+      <c r="N28" s="79" t="s">
+        <v>2</v>
+      </c>
       <c r="O28" s="85"/>
       <c r="P28" s="79"/>
       <c r="Q28" s="86"/>
@@ -9328,7 +9303,7 @@
       <c r="N29" s="79"/>
       <c r="O29" s="85"/>
       <c r="P29" s="79"/>
-      <c r="Q29" s="96"/>
+      <c r="Q29" s="97"/>
       <c r="R29" s="87" t="n">
         <f aca="false">IF(AND(C29="Normal",I29&gt;0),(8-S29),0)-IF(AND(C29="Normal",OR(C30="Special Holiday",C30="Working - Legal Holiday on RD",C30="Working - Special Holiday on RD",C30="Legal Holiday",C30="Legal Holiday on RD",C30="Special Holiday on RD")),BN29,0)+IF(AND(OR(C29="Normal",C29="Leave",C29="Rest Day"),OR(C28="Special Holiday",C28="Working - Legal Holiday on RD",C28="Working - Special Holiday on RD",C28="Legal Holiday")),BN28,0)</f>
         <v>0</v>
@@ -9776,7 +9751,7 @@
       <c r="N30" s="79"/>
       <c r="O30" s="85"/>
       <c r="P30" s="79"/>
-      <c r="Q30" s="97"/>
+      <c r="Q30" s="98"/>
       <c r="R30" s="87" t="n">
         <f aca="false">IF(AND(C30="Normal",I30&gt;0),(8-S30),0)-IF(AND(C30="Normal",OR(C31="Special Holiday",C31="Working - Legal Holiday on RD",C31="Working - Special Holiday on RD",C31="Legal Holiday",C31="Legal Holiday on RD",C31="Special Holiday on RD")),BN30,0)+IF(AND(OR(C30="Normal",C30="Leave",C30="Rest Day"),OR(C29="Special Holiday",C29="Working - Legal Holiday on RD",C29="Working - Special Holiday on RD",C29="Legal Holiday")),BN29,0)</f>
         <v>0</v>
@@ -10205,357 +10180,357 @@
       <c r="BY31" s="6"/>
     </row>
     <row r="32" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J32" s="98" t="s">
+      <c r="J32" s="99" t="s">
         <v>112</v>
       </c>
-      <c r="K32" s="98"/>
-      <c r="L32" s="98"/>
-      <c r="M32" s="98"/>
-      <c r="N32" s="99"/>
-      <c r="O32" s="99"/>
-      <c r="P32" s="99"/>
-      <c r="R32" s="100" t="n">
+      <c r="K32" s="99"/>
+      <c r="L32" s="99"/>
+      <c r="M32" s="99"/>
+      <c r="N32" s="100"/>
+      <c r="O32" s="100"/>
+      <c r="P32" s="100"/>
+      <c r="R32" s="101" t="n">
         <f aca="false">SUM(R14:R31)</f>
         <v>0</v>
       </c>
-      <c r="S32" s="100" t="n">
+      <c r="S32" s="101" t="n">
         <f aca="false">SUM(S14:S31)</f>
         <v>0</v>
       </c>
-      <c r="T32" s="100" t="n">
+      <c r="T32" s="101" t="n">
         <f aca="false">SUM(T14:T31)</f>
         <v>0</v>
       </c>
-      <c r="U32" s="100" t="n">
+      <c r="U32" s="101" t="n">
         <f aca="false">SUM(U14:U31)</f>
         <v>0</v>
       </c>
-      <c r="V32" s="100" t="n">
+      <c r="V32" s="101" t="n">
         <f aca="false">SUM(V14:V31)</f>
         <v>0</v>
       </c>
-      <c r="W32" s="100" t="n">
+      <c r="W32" s="101" t="n">
         <f aca="false">SUM(W14:W31)</f>
         <v>0</v>
       </c>
-      <c r="X32" s="100" t="n">
+      <c r="X32" s="101" t="n">
         <f aca="false">SUM(X14:X31)</f>
         <v>0</v>
       </c>
-      <c r="Y32" s="100" t="n">
+      <c r="Y32" s="101" t="n">
         <f aca="false">SUM(Y14:Y31)</f>
         <v>0</v>
       </c>
-      <c r="Z32" s="100" t="n">
+      <c r="Z32" s="101" t="n">
         <f aca="false">SUM(Z14:Z31)</f>
         <v>0</v>
       </c>
-      <c r="AA32" s="100" t="n">
+      <c r="AA32" s="101" t="n">
         <f aca="false">SUM(AA14:AA31)</f>
         <v>0</v>
       </c>
-      <c r="AB32" s="100" t="n">
+      <c r="AB32" s="101" t="n">
         <f aca="false">SUM(AB14:AB31)</f>
         <v>0</v>
       </c>
-      <c r="AC32" s="100" t="n">
+      <c r="AC32" s="101" t="n">
         <f aca="false">SUM(AC14:AC31)</f>
         <v>0</v>
       </c>
-      <c r="AD32" s="100" t="n">
+      <c r="AD32" s="101" t="n">
         <f aca="false">SUM(AD14:AD31)</f>
         <v>0</v>
       </c>
-      <c r="AE32" s="100" t="n">
+      <c r="AE32" s="101" t="n">
         <f aca="false">SUM(AE14:AE31)</f>
         <v>0</v>
       </c>
-      <c r="AF32" s="100" t="n">
+      <c r="AF32" s="101" t="n">
         <f aca="false">SUM(AF14:AF31)</f>
         <v>0</v>
       </c>
-      <c r="AG32" s="100" t="n">
+      <c r="AG32" s="101" t="n">
         <f aca="false">SUM(AG14:AG31)</f>
         <v>0</v>
       </c>
-      <c r="AH32" s="100" t="n">
+      <c r="AH32" s="101" t="n">
         <f aca="false">SUM(AH14:AH31)</f>
         <v>0</v>
       </c>
-      <c r="AI32" s="100" t="n">
+      <c r="AI32" s="101" t="n">
         <f aca="false">SUM(AI14:AI31)</f>
         <v>0</v>
       </c>
-      <c r="AJ32" s="100" t="n">
+      <c r="AJ32" s="101" t="n">
         <f aca="false">SUM(AJ14:AJ31)</f>
         <v>0</v>
       </c>
-      <c r="AK32" s="100" t="n">
+      <c r="AK32" s="101" t="n">
         <f aca="false">SUM(AK14:AK31)</f>
         <v>0</v>
       </c>
-      <c r="AL32" s="100" t="n">
+      <c r="AL32" s="101" t="n">
         <f aca="false">SUM(AL14:AL31)</f>
         <v>0</v>
       </c>
-      <c r="AM32" s="100" t="n">
+      <c r="AM32" s="101" t="n">
         <f aca="false">SUM(AM14:AM31)</f>
         <v>0</v>
       </c>
-      <c r="AN32" s="100" t="n">
+      <c r="AN32" s="101" t="n">
         <f aca="false">SUM(AN14:AN31)</f>
         <v>0</v>
       </c>
-      <c r="AO32" s="100" t="n">
+      <c r="AO32" s="101" t="n">
         <f aca="false">SUM(AO14:AO31)</f>
         <v>0</v>
       </c>
-      <c r="AP32" s="100" t="n">
+      <c r="AP32" s="101" t="n">
         <f aca="false">SUM(AP14:AP31)</f>
         <v>0</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M33" s="99"/>
-      <c r="N33" s="99"/>
-      <c r="O33" s="99"/>
-      <c r="P33" s="99"/>
-      <c r="R33" s="101"/>
-      <c r="S33" s="101"/>
-      <c r="T33" s="101"/>
-      <c r="U33" s="101"/>
-      <c r="V33" s="101"/>
-      <c r="W33" s="101"/>
-      <c r="X33" s="101"/>
-      <c r="Y33" s="101"/>
-      <c r="Z33" s="101"/>
-      <c r="AA33" s="101"/>
-      <c r="AB33" s="101"/>
-      <c r="AC33" s="101"/>
-      <c r="AD33" s="101"/>
-      <c r="AE33" s="101"/>
-      <c r="AF33" s="101"/>
-      <c r="AG33" s="101"/>
-      <c r="AH33" s="101"/>
-      <c r="AI33" s="101"/>
-      <c r="AJ33" s="101"/>
-      <c r="AK33" s="101"/>
-      <c r="AL33" s="101"/>
-      <c r="AM33" s="101"/>
-      <c r="AN33" s="101"/>
-      <c r="AO33" s="101"/>
-      <c r="AP33" s="101"/>
+      <c r="M33" s="100"/>
+      <c r="N33" s="100"/>
+      <c r="O33" s="100"/>
+      <c r="P33" s="100"/>
+      <c r="R33" s="102"/>
+      <c r="S33" s="102"/>
+      <c r="T33" s="102"/>
+      <c r="U33" s="102"/>
+      <c r="V33" s="102"/>
+      <c r="W33" s="102"/>
+      <c r="X33" s="102"/>
+      <c r="Y33" s="102"/>
+      <c r="Z33" s="102"/>
+      <c r="AA33" s="102"/>
+      <c r="AB33" s="102"/>
+      <c r="AC33" s="102"/>
+      <c r="AD33" s="102"/>
+      <c r="AE33" s="102"/>
+      <c r="AF33" s="102"/>
+      <c r="AG33" s="102"/>
+      <c r="AH33" s="102"/>
+      <c r="AI33" s="102"/>
+      <c r="AJ33" s="102"/>
+      <c r="AK33" s="102"/>
+      <c r="AL33" s="102"/>
+      <c r="AM33" s="102"/>
+      <c r="AN33" s="102"/>
+      <c r="AO33" s="102"/>
+      <c r="AP33" s="102"/>
     </row>
     <row r="34" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="102" t="s">
+      <c r="A34" s="103" t="s">
         <v>113</v>
       </c>
-      <c r="C34" s="103" t="s">
+      <c r="C34" s="104" t="s">
         <v>114</v>
       </c>
-      <c r="D34" s="103"/>
-      <c r="E34" s="103"/>
-      <c r="H34" s="102" t="s">
+      <c r="D34" s="104"/>
+      <c r="E34" s="104"/>
+      <c r="H34" s="103" t="s">
         <v>115</v>
       </c>
       <c r="I34" s="2"/>
-      <c r="K34" s="103" t="s">
+      <c r="K34" s="104" t="s">
         <v>12</v>
       </c>
-      <c r="L34" s="103"/>
-      <c r="M34" s="103"/>
-      <c r="N34" s="104"/>
+      <c r="L34" s="104"/>
+      <c r="M34" s="104"/>
+      <c r="N34" s="105"/>
     </row>
     <row r="35" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="102"/>
-      <c r="C35" s="105"/>
-      <c r="D35" s="105"/>
-      <c r="E35" s="105"/>
+      <c r="A35" s="103"/>
+      <c r="C35" s="106"/>
+      <c r="D35" s="106"/>
+      <c r="E35" s="106"/>
     </row>
     <row r="37" s="6" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="106" t="s">
+      <c r="A37" s="107" t="s">
         <v>116</v>
       </c>
-      <c r="B37" s="107" t="s">
+      <c r="B37" s="108" t="s">
         <v>99</v>
       </c>
-      <c r="C37" s="107" t="s">
+      <c r="C37" s="108" t="s">
         <v>100</v>
       </c>
-      <c r="D37" s="107" t="s">
+      <c r="D37" s="108" t="s">
         <v>101</v>
       </c>
-      <c r="E37" s="107" t="s">
+      <c r="E37" s="108" t="s">
         <v>117</v>
       </c>
-      <c r="F37" s="107" t="s">
+      <c r="F37" s="108" t="s">
         <v>56</v>
       </c>
       <c r="I37" s="9"/>
     </row>
-    <row r="38" s="110" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="108" t="s">
+    <row r="38" s="111" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="109" t="s">
         <v>99</v>
       </c>
-      <c r="B38" s="109" t="n">
+      <c r="B38" s="110" t="n">
         <f aca="false">R32+S32</f>
         <v>0</v>
       </c>
-      <c r="C38" s="109" t="n">
+      <c r="C38" s="110" t="n">
         <f aca="false">AK32</f>
         <v>0</v>
       </c>
-      <c r="D38" s="109" t="n">
+      <c r="D38" s="110" t="n">
         <f aca="false">Y32</f>
         <v>0</v>
       </c>
-      <c r="E38" s="109" t="n">
+      <c r="E38" s="110" t="n">
         <f aca="false">AE32</f>
         <v>0</v>
       </c>
-      <c r="F38" s="109" t="n">
+      <c r="F38" s="110" t="n">
         <f aca="false">S32</f>
         <v>0</v>
       </c>
-      <c r="I38" s="111"/>
+      <c r="I38" s="112"/>
     </row>
-    <row r="39" s="110" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="108" t="s">
+    <row r="39" s="111" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="109" t="s">
         <v>19</v>
       </c>
-      <c r="B39" s="109" t="n">
+      <c r="B39" s="110" t="n">
         <f aca="false">T32</f>
         <v>0</v>
       </c>
-      <c r="C39" s="109" t="n">
+      <c r="C39" s="110" t="n">
         <f aca="false">AL32</f>
         <v>0</v>
       </c>
-      <c r="D39" s="109" t="n">
+      <c r="D39" s="110" t="n">
         <f aca="false">Z32</f>
         <v>0</v>
       </c>
-      <c r="E39" s="109" t="n">
+      <c r="E39" s="110" t="n">
         <f aca="false">AF32</f>
         <v>0</v>
       </c>
-      <c r="F39" s="112" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" s="111"/>
+      <c r="F39" s="113" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="112"/>
     </row>
-    <row r="40" s="110" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="108" t="s">
+    <row r="40" s="111" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="109" t="s">
         <v>17</v>
       </c>
-      <c r="B40" s="109" t="n">
+      <c r="B40" s="110" t="n">
         <f aca="false">U32</f>
         <v>0</v>
       </c>
-      <c r="C40" s="109" t="n">
+      <c r="C40" s="110" t="n">
         <f aca="false">AM32</f>
         <v>0</v>
       </c>
-      <c r="D40" s="109" t="n">
+      <c r="D40" s="110" t="n">
         <f aca="false">AA32</f>
         <v>0</v>
       </c>
-      <c r="E40" s="109" t="n">
+      <c r="E40" s="110" t="n">
         <f aca="false">AG32</f>
         <v>0</v>
       </c>
-      <c r="F40" s="112" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" s="111"/>
+      <c r="F40" s="113" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="112"/>
     </row>
-    <row r="41" s="110" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="108" t="s">
+    <row r="41" s="111" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="109" t="s">
         <v>10</v>
       </c>
-      <c r="B41" s="109" t="n">
+      <c r="B41" s="110" t="n">
         <f aca="false">V32</f>
         <v>0</v>
       </c>
-      <c r="C41" s="109" t="n">
+      <c r="C41" s="110" t="n">
         <f aca="false">AN32</f>
         <v>0</v>
       </c>
-      <c r="D41" s="109" t="n">
+      <c r="D41" s="110" t="n">
         <f aca="false">AB32</f>
         <v>0</v>
       </c>
-      <c r="E41" s="109" t="n">
+      <c r="E41" s="110" t="n">
         <f aca="false">AH32</f>
         <v>0</v>
       </c>
-      <c r="F41" s="112" t="n">
-        <v>0</v>
-      </c>
-      <c r="I41" s="111"/>
+      <c r="F41" s="113" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="112"/>
     </row>
-    <row r="42" s="110" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="108" t="s">
+    <row r="42" s="111" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="109" t="s">
         <v>118</v>
       </c>
-      <c r="B42" s="109" t="n">
+      <c r="B42" s="110" t="n">
         <f aca="false">W32</f>
         <v>0</v>
       </c>
-      <c r="C42" s="109" t="n">
+      <c r="C42" s="110" t="n">
         <f aca="false">AO32</f>
         <v>0</v>
       </c>
-      <c r="D42" s="109" t="n">
+      <c r="D42" s="110" t="n">
         <f aca="false">AC32</f>
         <v>0</v>
       </c>
-      <c r="E42" s="109" t="n">
+      <c r="E42" s="110" t="n">
         <f aca="false">AI32</f>
         <v>0</v>
       </c>
-      <c r="F42" s="112" t="n">
-        <v>0</v>
-      </c>
-      <c r="I42" s="111"/>
+      <c r="F42" s="113" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="112"/>
     </row>
-    <row r="43" s="110" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="108" t="s">
+    <row r="43" s="111" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="109" t="s">
         <v>119</v>
       </c>
-      <c r="B43" s="109" t="n">
+      <c r="B43" s="110" t="n">
         <f aca="false">X32</f>
         <v>0</v>
       </c>
-      <c r="C43" s="109" t="n">
+      <c r="C43" s="110" t="n">
         <f aca="false">AP32</f>
         <v>0</v>
       </c>
-      <c r="D43" s="109" t="n">
+      <c r="D43" s="110" t="n">
         <f aca="false">AD32</f>
         <v>0</v>
       </c>
-      <c r="E43" s="109" t="n">
+      <c r="E43" s="110" t="n">
         <f aca="false">AJ32</f>
         <v>0</v>
       </c>
-      <c r="F43" s="112" t="n">
-        <v>0</v>
-      </c>
-      <c r="I43" s="111"/>
+      <c r="F43" s="113" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="112"/>
     </row>
     <row r="44" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="113" t="s">
+      <c r="A44" s="114" t="s">
         <v>120</v>
       </c>
-      <c r="B44" s="114" t="str">
+      <c r="B44" s="115" t="str">
         <f aca="false">COUNTIF(C14:C29,"Leave")&amp;" "&amp;"Leaves"&amp;" "&amp;"-"&amp;IF(C14="Leave",(TEXT(A14,"DD-mmm")&amp;","),"")&amp;" "&amp;IF(C15="Leave",(TEXT(A15,"DD-mmm")&amp;","),"")&amp;" "&amp;IF(C16="Leave",(TEXT(A16,"DD-mmm")&amp;","),"")&amp;" "&amp;IF(C17="Leave",(TEXT(A17,"DD-mmm")&amp;","),"")&amp;" "&amp;IF(C18="Leave",(TEXT(A18,"DD-mmm")&amp;","),"")&amp;" "&amp;IF(C19="Leave",(TEXT(A19,"DD-mmm")&amp;","),"")&amp;" "&amp;IF(C20="Leave",(TEXT(A20,"DD-mmm")&amp;","),"")&amp;" "&amp;IF(C21="Leave",(TEXT(A21,"DD-mmm")&amp;","),"")&amp;" "&amp;IF(C22="Leave",(TEXT(A22,"DD-mmm")&amp;","),"")&amp;" "&amp;IF(C23="Leave",(TEXT(A23,"DD-mmm")&amp;","),"")&amp;" "&amp;IF(C24="Leave",(TEXT(A24,"DD-mmm")&amp;","),"")&amp;" "&amp;IF(C25="Leave",(TEXT(A25,"DD-mmm")&amp;","),"")&amp;" "&amp;IF(C26="Leave",(TEXT(A26,"DD-mmm")&amp;","),"")&amp;" "&amp;IF(C27="Leave",(TEXT(A27,"DD-mmm")&amp;","),"")&amp;" "&amp;IF(C28="Leave",(TEXT(A28,"DD-mmm")&amp;","),"")&amp;" "&amp;IF(C29="Leave",(TEXT(A29,"DD-mmm")&amp;","),"")</f>
         <v>2 Leaves -   19-Jan,       26-Jan,     </v>
       </c>
-      <c r="C44" s="114"/>
-      <c r="D44" s="114"/>
-      <c r="E44" s="114"/>
-      <c r="F44" s="114"/>
+      <c r="C44" s="115"/>
+      <c r="D44" s="115"/>
+      <c r="E44" s="115"/>
+      <c r="F44" s="115"/>
     </row>
   </sheetData>
   <sheetProtection sheet="true" password="d9ff" formatCells="false" formatColumns="false" formatRows="false" autoFilter="false" pivotTables="false"/>
@@ -10602,10 +10577,10 @@
     <mergeCell ref="B44:F44"/>
   </mergeCells>
   <conditionalFormatting sqref="B14:B30">
-    <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Sun" dxfId="6">
+    <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Sun" dxfId="0">
       <formula>NOT(ISERROR(SEARCH("Sun",B14)))</formula>
     </cfRule>
-    <cfRule type="containsText" priority="3" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Sat" dxfId="7">
+    <cfRule type="containsText" priority="3" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Sat" dxfId="1">
       <formula>NOT(ISERROR(SEARCH("Sat",B14)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>